<commit_message>
cambio de la competencia de Comunicacion
</commit_message>
<xml_diff>
--- a/public/plantillas/COMUNICACION_SE_COMUNICA.xlsx
+++ b/public/plantillas/COMUNICACION_SE_COMUNICA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO\Desktop\xds\PROYECTOS\inicial-notas\public\plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF5B00C3-FBBE-48B3-9BF6-8C3EB81BFD00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC156139-BC8E-4B43-9A04-B6348BF01F2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,9 +42,6 @@
     <t>crierio de evaluacion</t>
   </si>
   <si>
-    <t>Se comunica oralmente mediante diversos tipos de textos; identifica información explícita; realiza inferencias sencillas a partir de esta información e interpreta recursos no verbales y paraverbales de las personas de su entorno. Opina sobre lo que más/menos le gustó del contenido del texto. Se expresa espontáneamente a partir de sus conocimientos previos, con el propósito de interactuar con uno o más interlocutores conocidos en una situación comunicativa. Desarrolla sus ideas manteniéndose por lo general en el tema; utiliza vocabulario de uso frecuente y una pronunciación entendible, se apoya en gestos y lenguaje corporal. En un intercambio, generalmente participa y responde en forma pertinente a lo que le dicen</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 	Obtiene información del texto oral.                    
  	Infiere e interpreta información del texto oral.  
  	Adecúa, organiza y desarrolla las ideas de forma coherente y cohesionada.             
@@ -143,12 +140,15 @@
   <si>
     <t>ACTIVIDAD:</t>
   </si>
+  <si>
+    <t>SE COMUNICA ORALMENTE EN SU LENGUA MATERNA Se comunica oralmente mediante diversos tipos de textos; identifica información explícita; realiza inferencias sencillas a partir de esta información e interpreta recursos no verbales y paraverbales de las personas de su entorno. Opina sobre lo que más/menos le gustó del contenido del texto. Se expresa espontáneamente a partir de sus conocimientos previos, con el propósito de interactuar con uno o más interlocutores conocidos en una situación comunicativa. Desarrolla sus ideas manteniéndose por lo general en el tema; utiliza vocabulario de uso frecuente y una pronunciación entendible, se apoya en gestos y lenguaje corporal. En un intercambio, generalmente participa y responde en forma pertinente a lo que le dicen</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -196,6 +196,12 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -270,7 +276,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -290,29 +296,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -324,6 +312,27 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -553,245 +562,245 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="10"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="11"/>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="11"/>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="11"/>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="11"/>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" s="21" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="10"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="11"/>
+      <c r="F5" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="G5" s="10"/>
+      <c r="H5" s="11"/>
+    </row>
+    <row r="6" spans="1:8" ht="171.75" customHeight="1">
+      <c r="A6" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="10"/>
-    </row>
-    <row r="3" spans="1:8">
-      <c r="A3" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="B3" s="11"/>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="10"/>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="11"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="10"/>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" s="13" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" s="11"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="13" t="s">
-        <v>3</v>
-      </c>
-      <c r="E5" s="10"/>
-      <c r="F5" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="G5" s="11"/>
-      <c r="H5" s="10"/>
-    </row>
-    <row r="6" spans="1:8" ht="171.75" customHeight="1">
-      <c r="A6" s="9" t="s">
+      <c r="B6" s="10"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="11"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="9" t="s">
+      <c r="E6" s="11"/>
+      <c r="F6" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="10"/>
-      <c r="F6" s="9" t="s">
+      <c r="G6" s="10"/>
+      <c r="H6" s="11"/>
+    </row>
+    <row r="7" spans="1:8" ht="17.25">
+      <c r="A7" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="11"/>
-      <c r="H6" s="10"/>
-    </row>
-    <row r="7" spans="1:8" ht="17.25">
-      <c r="A7" s="14" t="s">
+      <c r="B7" s="10"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="11"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="H7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H7" s="1" t="s">
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" s="18" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="8" spans="1:8">
-      <c r="A8" s="15" t="s">
+      <c r="B8" s="10"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="11"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="F8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>17</v>
-      </c>
       <c r="H8" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="35.25" customHeight="1">
       <c r="A9" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="B9" s="11"/>
-      <c r="C9" s="10"/>
+        <v>17</v>
+      </c>
+      <c r="B9" s="10"/>
+      <c r="C9" s="11"/>
       <c r="D9" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E9" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F9" s="3" t="s">
+      <c r="H9" s="2" t="s">
         <v>15</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="28.5" customHeight="1">
       <c r="A10" s="16" t="s">
-        <v>19</v>
-      </c>
-      <c r="B10" s="11"/>
-      <c r="C10" s="10"/>
+        <v>18</v>
+      </c>
+      <c r="B10" s="10"/>
+      <c r="C10" s="11"/>
       <c r="D10" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F10" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F10" s="3" t="s">
+      <c r="G10" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G10" s="3" t="s">
-        <v>17</v>
-      </c>
       <c r="H10" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="24.75" customHeight="1">
       <c r="A11" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="B11" s="11"/>
-      <c r="C11" s="10"/>
+        <v>19</v>
+      </c>
+      <c r="B11" s="10"/>
+      <c r="C11" s="11"/>
       <c r="D11" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="3" t="s">
-        <v>16</v>
-      </c>
       <c r="F11" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G11" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="G11" s="3" t="s">
-        <v>16</v>
-      </c>
       <c r="H11" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="26.25" customHeight="1">
       <c r="A12" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="B12" s="11"/>
-      <c r="C12" s="10"/>
+        <v>20</v>
+      </c>
+      <c r="B12" s="10"/>
+      <c r="C12" s="11"/>
       <c r="D12" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E12" s="3" t="s">
-        <v>16</v>
-      </c>
       <c r="F12" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="G12" s="3" t="s">
-        <v>16</v>
-      </c>
       <c r="H12" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="31.5" customHeight="1">
       <c r="A13" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" s="11"/>
-      <c r="C13" s="10"/>
+        <v>21</v>
+      </c>
+      <c r="B13" s="10"/>
+      <c r="C13" s="11"/>
       <c r="D13" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E13" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E13" s="3" t="s">
-        <v>17</v>
-      </c>
       <c r="F13" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="G13" s="3" t="s">
-        <v>16</v>
-      </c>
       <c r="H13" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="24" customHeight="1">
-      <c r="A14" s="18" t="s">
-        <v>22</v>
-      </c>
-      <c r="B14" s="11"/>
-      <c r="C14" s="10"/>
+      <c r="A14" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" s="10"/>
+      <c r="C14" s="11"/>
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
@@ -799,11 +808,11 @@
       <c r="H14" s="5"/>
     </row>
     <row r="15" spans="1:8" ht="25.5" customHeight="1">
-      <c r="A15" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="B15" s="11"/>
-      <c r="C15" s="10"/>
+      <c r="A15" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" s="10"/>
+      <c r="C15" s="11"/>
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
@@ -811,11 +820,11 @@
       <c r="H15" s="5"/>
     </row>
     <row r="16" spans="1:8" ht="33" customHeight="1">
-      <c r="A16" s="18" t="s">
-        <v>24</v>
-      </c>
-      <c r="B16" s="11"/>
-      <c r="C16" s="10"/>
+      <c r="A16" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" s="10"/>
+      <c r="C16" s="11"/>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
@@ -823,28 +832,28 @@
       <c r="H16" s="5"/>
     </row>
     <row r="17" spans="1:8" ht="23.25" customHeight="1">
-      <c r="A17" s="19" t="s">
+      <c r="A17" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17" s="10"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="11"/>
+    </row>
+    <row r="19" spans="1:8" ht="15.75">
+      <c r="A19" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="11"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="11"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="10"/>
-    </row>
-    <row r="19" spans="1:8" ht="15.75">
-      <c r="A19" s="20" t="s">
-        <v>26</v>
-      </c>
-      <c r="B19" s="11"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="11"/>
-      <c r="H19" s="10"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="11"/>
     </row>
     <row r="20" spans="1:8">
       <c r="A20" s="6"/>
@@ -858,89 +867,89 @@
     </row>
     <row r="21" spans="1:8">
       <c r="A21" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="C21" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="C21" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="11"/>
-      <c r="H21" s="10"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="10"/>
+      <c r="G21" s="10"/>
+      <c r="H21" s="11"/>
     </row>
     <row r="22" spans="1:8" ht="63.75" customHeight="1">
       <c r="A22" s="8"/>
       <c r="B22" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C22" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="10"/>
+        <v>14</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D22" s="10"/>
+      <c r="E22" s="10"/>
+      <c r="F22" s="10"/>
+      <c r="G22" s="10"/>
+      <c r="H22" s="11"/>
     </row>
     <row r="23" spans="1:8" ht="63" customHeight="1">
       <c r="A23" s="8"/>
       <c r="B23" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C23" s="17" t="s">
-        <v>31</v>
-      </c>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="11"/>
-      <c r="G23" s="11"/>
-      <c r="H23" s="10"/>
+        <v>15</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="D23" s="10"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="11"/>
     </row>
     <row r="24" spans="1:8" ht="46.5" customHeight="1">
       <c r="A24" s="8"/>
       <c r="B24" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C24" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="D24" s="11"/>
-      <c r="E24" s="11"/>
-      <c r="F24" s="11"/>
-      <c r="G24" s="11"/>
-      <c r="H24" s="10"/>
+        <v>14</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D24" s="10"/>
+      <c r="E24" s="10"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="10"/>
+      <c r="H24" s="11"/>
     </row>
     <row r="25" spans="1:8" ht="47.25" customHeight="1">
       <c r="A25" s="8"/>
       <c r="B25" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C25" s="17" t="s">
-        <v>33</v>
-      </c>
-      <c r="D25" s="11"/>
-      <c r="E25" s="11"/>
-      <c r="F25" s="11"/>
-      <c r="G25" s="11"/>
-      <c r="H25" s="10"/>
+        <v>16</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="D25" s="10"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="10"/>
+      <c r="H25" s="11"/>
     </row>
     <row r="26" spans="1:8" ht="48.75" customHeight="1">
       <c r="A26" s="8"/>
       <c r="B26" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C26" s="17" t="s">
-        <v>34</v>
-      </c>
-      <c r="D26" s="11"/>
-      <c r="E26" s="11"/>
-      <c r="F26" s="11"/>
-      <c r="G26" s="11"/>
-      <c r="H26" s="10"/>
+        <v>15</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D26" s="10"/>
+      <c r="E26" s="10"/>
+      <c r="F26" s="10"/>
+      <c r="G26" s="10"/>
+      <c r="H26" s="11"/>
     </row>
     <row r="27" spans="1:8" ht="15.75" customHeight="1"/>
     <row r="28" spans="1:8" ht="15.75" customHeight="1"/>
@@ -1919,24 +1928,6 @@
     <row r="1001" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="C26:H26"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="A16:C16"/>
-    <mergeCell ref="A17:H17"/>
-    <mergeCell ref="A19:H19"/>
-    <mergeCell ref="C21:H21"/>
-    <mergeCell ref="C22:H22"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="C23:H23"/>
-    <mergeCell ref="C24:H24"/>
-    <mergeCell ref="C25:H25"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A11:C11"/>
     <mergeCell ref="D6:E6"/>
     <mergeCell ref="F6:H6"/>
     <mergeCell ref="A1:H1"/>
@@ -1947,6 +1938,24 @@
     <mergeCell ref="F5:H5"/>
     <mergeCell ref="A6:C6"/>
     <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="C23:H23"/>
+    <mergeCell ref="C24:H24"/>
+    <mergeCell ref="C25:H25"/>
+    <mergeCell ref="C26:H26"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="A17:H17"/>
+    <mergeCell ref="A19:H19"/>
+    <mergeCell ref="C21:H21"/>
+    <mergeCell ref="C22:H22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>